<commit_message>
data: scanner sync 2026-09-29 20:47
</commit_message>
<xml_diff>
--- a/data/kq_scan_results.xlsx
+++ b/data/kq_scan_results.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -599,19 +599,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>61.42</v>
+        <v>86.25</v>
       </c>
       <c r="D2" t="n">
         <v>32.35</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>89.86</v>
+        <v>166.62</v>
       </c>
       <c r="F2" t="n">
-        <v>5466753</v>
+        <v>81530</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2903.6</v>
+        <v>43.3</v>
       </c>
       <c r="H2" t="n">
         <v>1882</v>
@@ -638,19 +638,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5.87</v>
+        <v>4.35</v>
       </c>
       <c r="D3" t="n">
         <v>3.45</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>70.14</v>
+        <v>26.09</v>
       </c>
       <c r="F3" t="n">
-        <v>14766975</v>
+        <v>114285</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>20407.6</v>
+        <v>157.9</v>
       </c>
       <c r="H3" t="n">
         <v>723</v>
@@ -673,36 +673,36 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AMPX</t>
+          <t>YDES</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11.2</v>
+        <v>7.1</v>
       </c>
       <c r="D4" t="n">
-        <v>9.75</v>
+        <v>5.73</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>14.87</v>
+        <v>23.91</v>
       </c>
       <c r="F4" t="n">
-        <v>2005979</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>102.6</v>
+        <v>745</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>19559</v>
+        <v>301952</v>
       </c>
       <c r="I4" t="n">
-        <v>5219558</v>
+        <v>301952</v>
       </c>
       <c r="J4" t="n">
-        <v>4.54</v>
+        <v>22.01</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>pm</t>
+          <t>proxy</t>
         </is>
       </c>
     </row>
@@ -712,34 +712,424 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FIGS</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14.5</v>
+        <v>18.49</v>
       </c>
       <c r="D5" t="n">
-        <v>13.42</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>8.050000000000001</v>
+        <v>15.61</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>18.45</v>
       </c>
       <c r="F5" t="n">
-        <v>13592</v>
+        <v>855574</v>
       </c>
       <c r="G5" s="2" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="H5" t="n">
+        <v>18621</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5441086</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ABCL</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>14.28</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="F6" t="n">
+        <v>77937</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>38884</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6836784</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5.52</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AGEN</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8052</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10954</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1319892</v>
+      </c>
+      <c r="J7" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CBIO</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>15.67</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1461</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>31</v>
+      </c>
+      <c r="I8" t="n">
+        <v>362400</v>
+      </c>
+      <c r="J8" t="n">
+        <v>8.619999999999999</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>12.13</v>
+      </c>
+      <c r="D9" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="F9" t="n">
+        <v>495805</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H9" t="n">
+        <v>56955</v>
+      </c>
+      <c r="I9" t="n">
+        <v>16483104</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="D10" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5193</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>774</v>
+      </c>
+      <c r="I10" t="n">
+        <v>571830</v>
+      </c>
+      <c r="J10" t="n">
         <v>6.2</v>
       </c>
-      <c r="H5" t="n">
-        <v>2189</v>
-      </c>
-      <c r="I5" t="n">
-        <v>2909368</v>
-      </c>
-      <c r="J5" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>VOYG</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>34.41</v>
+      </c>
+      <c r="D11" t="n">
+        <v>31.35</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="F11" t="n">
+        <v>25621</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1492</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1845858</v>
+      </c>
+      <c r="J11" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="D12" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="F12" t="n">
+        <v>300</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1062</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1361720</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IRD</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6862</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>29312</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2613568</v>
+      </c>
+      <c r="J13" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3068</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1955</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1164750</v>
+      </c>
+      <c r="J14" t="n">
+        <v>5.52</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>XERS</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="D15" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2137</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="H15" t="n">
+        <v>362</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1744940</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t>pm</t>
         </is>
@@ -16501,7 +16891,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-09-29 12:16:38</t>
+          <t>2026-09-29 20:46:37</t>
         </is>
       </c>
     </row>
@@ -16522,7 +16912,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -16603,7 +16993,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>405s</t>
+          <t>94s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: scanner sync 2026-10-22 20:52
</commit_message>
<xml_diff>
--- a/data/kq_scan_results.xlsx
+++ b/data/kq_scan_results.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -595,36 +595,36 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SAIQ</t>
+          <t>BHVN</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5.88</v>
+        <v>15.8</v>
       </c>
       <c r="D2" t="n">
-        <v>3.41</v>
+        <v>11.81</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>72.43000000000001</v>
+        <v>33.78</v>
       </c>
       <c r="F2" t="n">
-        <v>603849</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>0.3</v>
+        <v>4861804</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>185.8</v>
       </c>
       <c r="H2" t="n">
-        <v>2057624</v>
+        <v>26165</v>
       </c>
       <c r="I2" t="n">
-        <v>2057624</v>
+        <v>2839838</v>
       </c>
       <c r="J2" t="n">
-        <v>28.52</v>
+        <v>5.7</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>proxy</t>
+          <t>pm</t>
         </is>
       </c>
     </row>
@@ -634,32 +634,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>BETR</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>45.46</v>
+        <v>14.88</v>
       </c>
       <c r="D3" t="n">
-        <v>30.04</v>
+        <v>11.97</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>51.33</v>
+        <v>24.31</v>
       </c>
       <c r="F3" t="n">
-        <v>7835</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>0.3</v>
+        <v>7139</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>5.5</v>
       </c>
       <c r="H3" t="n">
-        <v>30872</v>
+        <v>1306</v>
       </c>
       <c r="I3" t="n">
-        <v>2519070</v>
+        <v>772776</v>
       </c>
       <c r="J3" t="n">
-        <v>5.18</v>
+        <v>11.24</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -673,32 +673,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MYGN</t>
+          <t>AMTD</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5.66</v>
+        <v>30</v>
       </c>
       <c r="D4" t="n">
-        <v>4.21</v>
+        <v>24.78</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>34.44</v>
+        <v>21.07</v>
       </c>
       <c r="F4" t="n">
-        <v>30086</v>
+        <v>10</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1825502</v>
+        <v>1790636</v>
       </c>
       <c r="I4" t="n">
-        <v>1825502</v>
+        <v>1790636</v>
       </c>
       <c r="J4" t="n">
-        <v>6.28</v>
+        <v>14.26</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -712,32 +712,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BNC</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5.69</v>
+        <v>22</v>
       </c>
       <c r="D5" t="n">
-        <v>4.67</v>
+        <v>19.04</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>21.84</v>
+        <v>15.55</v>
       </c>
       <c r="F5" t="n">
-        <v>62385</v>
+        <v>1348</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="H5" t="n">
-        <v>318679</v>
+        <v>5246</v>
       </c>
       <c r="I5" t="n">
-        <v>2577928</v>
+        <v>793500</v>
       </c>
       <c r="J5" t="n">
-        <v>5.09</v>
+        <v>7.64</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -751,32 +751,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CTNM</t>
+          <t>AMRC</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8.800000000000001</v>
+        <v>21.5</v>
       </c>
       <c r="D6" t="n">
-        <v>7.44</v>
+        <v>18.75</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>18.28</v>
+        <v>14.67</v>
       </c>
       <c r="F6" t="n">
-        <v>863</v>
+        <v>1224</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0.7</v>
       </c>
       <c r="H6" t="n">
-        <v>1284</v>
+        <v>1712</v>
       </c>
       <c r="I6" t="n">
-        <v>895242</v>
+        <v>638218</v>
       </c>
       <c r="J6" t="n">
-        <v>10.44</v>
+        <v>4.88</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -790,32 +790,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BETR</t>
+          <t>VERX</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>12.33</v>
+        <v>16</v>
       </c>
       <c r="D7" t="n">
-        <v>10.53</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>17.09</v>
+        <v>14.32</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>11.73</v>
       </c>
       <c r="F7" t="n">
-        <v>1592</v>
+        <v>202</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>1.2</v>
+        <v>0.1</v>
       </c>
       <c r="H7" t="n">
-        <v>1291</v>
+        <v>1957</v>
       </c>
       <c r="I7" t="n">
-        <v>772776</v>
+        <v>1477930</v>
       </c>
       <c r="J7" t="n">
-        <v>11.24</v>
+        <v>4.19</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -829,36 +829,36 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SLE</t>
+          <t>RCEL</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5.62</v>
+        <v>15.41</v>
       </c>
       <c r="D8" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>17.08</v>
+        <v>13.8</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>11.68</v>
       </c>
       <c r="F8" t="n">
-        <v>1722</v>
+        <v>156</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="H8" t="n">
-        <v>1681546</v>
+        <v>242</v>
       </c>
       <c r="I8" t="n">
-        <v>1681546</v>
+        <v>374566</v>
       </c>
       <c r="J8" t="n">
-        <v>8.84</v>
+        <v>5.77</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>proxy</t>
+          <t>pm</t>
         </is>
       </c>
     </row>
@@ -868,32 +868,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SLS</t>
+          <t>APPN</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>12.04</v>
+        <v>49</v>
       </c>
       <c r="D9" t="n">
-        <v>10.49</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>14.78</v>
+        <v>44.51</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>10.09</v>
       </c>
       <c r="F9" t="n">
-        <v>44915</v>
+        <v>2329</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.8</v>
+        <v>2.1</v>
       </c>
       <c r="H9" t="n">
-        <v>57080</v>
+        <v>1103</v>
       </c>
       <c r="I9" t="n">
-        <v>6537934</v>
+        <v>850976</v>
       </c>
       <c r="J9" t="n">
-        <v>6.56</v>
+        <v>5.79</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -907,32 +907,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PAY</t>
+          <t>ALMR</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D10" t="n">
-        <v>31.44</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>14.5</v>
+        <v>28.16</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>10.08</v>
       </c>
       <c r="F10" t="n">
-        <v>107</v>
+        <v>27</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H10" t="n">
-        <v>878</v>
+        <v>172</v>
       </c>
       <c r="I10" t="n">
-        <v>1055012</v>
+        <v>544326</v>
       </c>
       <c r="J10" t="n">
-        <v>4.02</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -946,36 +946,36 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DUOT</t>
+          <t>SKYD</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6.27</v>
+        <v>7.78</v>
       </c>
       <c r="D11" t="n">
-        <v>5.48</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>14.44</v>
+        <v>7.1</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>9.51</v>
       </c>
       <c r="F11" t="n">
-        <v>13891</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>5.9</v>
+        <v>2285114</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0.1</v>
       </c>
       <c r="H11" t="n">
-        <v>2336</v>
+        <v>23469770</v>
       </c>
       <c r="I11" t="n">
-        <v>1020586</v>
+        <v>23469770</v>
       </c>
       <c r="J11" t="n">
-        <v>6.57</v>
+        <v>7.04</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>pm</t>
+          <t>proxy</t>
         </is>
       </c>
     </row>
@@ -985,32 +985,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TRAX</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>41.5</v>
+        <v>21.7</v>
       </c>
       <c r="D12" t="n">
-        <v>36.28</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>14.39</v>
+        <v>19.82</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>9.49</v>
       </c>
       <c r="F12" t="n">
-        <v>726</v>
+        <v>14815</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="H12" t="n">
-        <v>3703</v>
+        <v>11637</v>
       </c>
       <c r="I12" t="n">
-        <v>875620</v>
+        <v>6463650</v>
       </c>
       <c r="J12" t="n">
-        <v>8.75</v>
+        <v>5.3</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1024,32 +1024,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>KLRA</t>
+          <t>AIP</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>13</v>
+        <v>21.5</v>
       </c>
       <c r="D13" t="n">
-        <v>11.43</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>13.74</v>
+        <v>19.76</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>8.81</v>
       </c>
       <c r="F13" t="n">
-        <v>45</v>
+        <v>139</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H13" t="n">
-        <v>187</v>
+        <v>1640</v>
       </c>
       <c r="I13" t="n">
-        <v>1100206</v>
+        <v>674928</v>
       </c>
       <c r="J13" t="n">
-        <v>7.9</v>
+        <v>4.56</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1063,32 +1063,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>GRRR</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>36.5</v>
+        <v>8.09</v>
       </c>
       <c r="D14" t="n">
-        <v>32.1</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>13.71</v>
+        <v>7.44</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>8.68</v>
       </c>
       <c r="F14" t="n">
-        <v>2338361</v>
+        <v>37279</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>5.9</v>
+        <v>7</v>
       </c>
       <c r="H14" t="n">
-        <v>393111</v>
+        <v>5349</v>
       </c>
       <c r="I14" t="n">
-        <v>43332198</v>
+        <v>959052</v>
       </c>
       <c r="J14" t="n">
-        <v>5.28</v>
+        <v>7.65</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1102,32 +1102,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FRNM</t>
+          <t>SWMR</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.24</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>12.57</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>13.29</v>
+        <v>9.029999999999999</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>8.59</v>
       </c>
       <c r="F15" t="n">
-        <v>168</v>
+        <v>3415</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H15" t="n">
-        <v>431</v>
+        <v>5542</v>
       </c>
       <c r="I15" t="n">
-        <v>899838</v>
+        <v>741786</v>
       </c>
       <c r="J15" t="n">
-        <v>7.04</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1141,36 +1141,36 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BIOA</t>
+          <t>CRL</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5.65</v>
+        <v>342.5</v>
       </c>
       <c r="D16" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>13.27</v>
+        <v>315.45</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>8.58</v>
       </c>
       <c r="F16" t="n">
-        <v>116</v>
+        <v>439</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>1430</v>
+        <v>941068</v>
       </c>
       <c r="I16" t="n">
-        <v>725348</v>
+        <v>941068</v>
       </c>
       <c r="J16" t="n">
-        <v>6.27</v>
+        <v>4.06</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>pm</t>
+          <t>proxy</t>
         </is>
       </c>
     </row>
@@ -1180,2064 +1180,36 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>USDE</t>
+          <t>NET</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>11.52</v>
+        <v>315.9</v>
       </c>
       <c r="D17" t="n">
-        <v>10.21</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>12.79</v>
+        <v>291.69</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>8.300000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>46552</v>
-      </c>
-      <c r="G17" s="3" t="n">
-        <v>0.4</v>
+        <v>40472</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>4.9</v>
       </c>
       <c r="H17" t="n">
-        <v>126407</v>
+        <v>8294</v>
       </c>
       <c r="I17" t="n">
-        <v>6048062</v>
+        <v>3224498</v>
       </c>
       <c r="J17" t="n">
-        <v>10.54</v>
+        <v>4.52</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>NESR</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="D18" t="n">
-        <v>18.98</v>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>12.22</v>
-      </c>
-      <c r="F18" t="n">
-        <v>926</v>
-      </c>
-      <c r="G18" s="3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H18" t="n">
-        <v>1494</v>
-      </c>
-      <c r="I18" t="n">
-        <v>2431654</v>
-      </c>
-      <c r="J18" t="n">
-        <v>5.69</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SSMR</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>13</v>
-      </c>
-      <c r="D19" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>12.07</v>
-      </c>
-      <c r="F19" t="n">
-        <v>60</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H19" t="n">
-        <v>369</v>
-      </c>
-      <c r="I19" t="n">
-        <v>442754</v>
-      </c>
-      <c r="J19" t="n">
-        <v>5.54</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>EQPT</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="D20" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>11.83</v>
-      </c>
-      <c r="F20" t="n">
-        <v>111</v>
-      </c>
-      <c r="G20" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1391</v>
-      </c>
-      <c r="I20" t="n">
-        <v>3288242</v>
-      </c>
-      <c r="J20" t="n">
-        <v>8.24</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>RUN</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="D21" t="n">
-        <v>6.89</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>11.76</v>
-      </c>
-      <c r="F21" t="n">
-        <v>15908</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H21" t="n">
-        <v>20584</v>
-      </c>
-      <c r="I21" t="n">
-        <v>7748080</v>
-      </c>
-      <c r="J21" t="n">
-        <v>4.92</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>DFH</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>9.640000000000001</v>
-      </c>
-      <c r="D22" t="n">
-        <v>8.65</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>11.45</v>
-      </c>
-      <c r="F22" t="n">
-        <v>1118</v>
-      </c>
-      <c r="G22" s="3" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H22" t="n">
-        <v>646</v>
-      </c>
-      <c r="I22" t="n">
-        <v>1109662</v>
-      </c>
-      <c r="J22" t="n">
-        <v>6.66</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>ATEC</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="D23" t="n">
-        <v>10.41</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>11.43</v>
-      </c>
-      <c r="F23" t="n">
-        <v>12863</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H23" t="n">
-        <v>6093</v>
-      </c>
-      <c r="I23" t="n">
-        <v>2062360</v>
-      </c>
-      <c r="J23" t="n">
-        <v>4.41</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>ADUR</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>11</v>
-      </c>
-      <c r="D24" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>11.11</v>
-      </c>
-      <c r="F24" t="n">
-        <v>3396</v>
-      </c>
-      <c r="G24" s="3" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="H24" t="n">
-        <v>2643</v>
-      </c>
-      <c r="I24" t="n">
-        <v>337740</v>
-      </c>
-      <c r="J24" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>OBX</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>13.25</v>
-      </c>
-      <c r="D25" t="n">
-        <v>11.94</v>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>10.97</v>
-      </c>
-      <c r="F25" t="n">
-        <v>219</v>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>433818</v>
-      </c>
-      <c r="I25" t="n">
-        <v>433818</v>
-      </c>
-      <c r="J25" t="n">
-        <v>9.869999999999999</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>proxy</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>KVYO</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>19.43</v>
-      </c>
-      <c r="D26" t="n">
-        <v>17.52</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>10.91</v>
-      </c>
-      <c r="F26" t="n">
-        <v>136164</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="H26" t="n">
-        <v>16664</v>
-      </c>
-      <c r="I26" t="n">
-        <v>5977442</v>
-      </c>
-      <c r="J26" t="n">
-        <v>5.34</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>GRML</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>6.21</v>
-      </c>
-      <c r="D27" t="n">
-        <v>5.61</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="F27" t="n">
-        <v>19969</v>
-      </c>
-      <c r="G27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" t="n">
-        <v>1221992</v>
-      </c>
-      <c r="I27" t="n">
-        <v>11082471</v>
-      </c>
-      <c r="J27" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>SGMT</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="D28" t="n">
-        <v>8.859999999999999</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>10.61</v>
-      </c>
-      <c r="F28" t="n">
-        <v>7238</v>
-      </c>
-      <c r="G28" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H28" t="n">
-        <v>14817</v>
-      </c>
-      <c r="I28" t="n">
-        <v>1341592</v>
-      </c>
-      <c r="J28" t="n">
-        <v>7.34</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ARQQ</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="D29" t="n">
-        <v>14.02</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>10.56</v>
-      </c>
-      <c r="F29" t="n">
-        <v>763</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H29" t="n">
-        <v>2960</v>
-      </c>
-      <c r="I29" t="n">
-        <v>326648</v>
-      </c>
-      <c r="J29" t="n">
-        <v>8.44</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>OPTX</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>7.34</v>
-      </c>
-      <c r="D30" t="n">
-        <v>6.64</v>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>10.54</v>
-      </c>
-      <c r="F30" t="n">
-        <v>237</v>
-      </c>
-      <c r="G30" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H30" t="n">
-        <v>1380</v>
-      </c>
-      <c r="I30" t="n">
-        <v>345490</v>
-      </c>
-      <c r="J30" t="n">
-        <v>7.66</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>QTTB</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="D31" t="n">
-        <v>7.79</v>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>10.53</v>
-      </c>
-      <c r="F31" t="n">
-        <v>624</v>
-      </c>
-      <c r="G31" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H31" t="n">
-        <v>8317</v>
-      </c>
-      <c r="I31" t="n">
-        <v>777734</v>
-      </c>
-      <c r="J31" t="n">
-        <v>8.529999999999999</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>EPRX</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>7.67</v>
-      </c>
-      <c r="D32" t="n">
-        <v>6.95</v>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>10.36</v>
-      </c>
-      <c r="F32" t="n">
-        <v>11</v>
-      </c>
-      <c r="G32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" t="n">
-        <v>225</v>
-      </c>
-      <c r="I32" t="n">
-        <v>678254</v>
-      </c>
-      <c r="J32" t="n">
-        <v>7.18</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>HTFL</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>56.23</v>
-      </c>
-      <c r="D33" t="n">
-        <v>51.02</v>
-      </c>
-      <c r="E33" s="3" t="n">
-        <v>10.22</v>
-      </c>
-      <c r="F33" t="n">
-        <v>5632</v>
-      </c>
-      <c r="G33" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H33" t="n">
-        <v>3095</v>
-      </c>
-      <c r="I33" t="n">
-        <v>2075378</v>
-      </c>
-      <c r="J33" t="n">
-        <v>5.41</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>ARVN</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>8</v>
-      </c>
-      <c r="D34" t="n">
-        <v>7.26</v>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>10.17</v>
-      </c>
-      <c r="F34" t="n">
-        <v>315</v>
-      </c>
-      <c r="G34" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H34" t="n">
-        <v>989</v>
-      </c>
-      <c r="I34" t="n">
-        <v>739524</v>
-      </c>
-      <c r="J34" t="n">
-        <v>4.69</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>NAMS</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>22.55</v>
-      </c>
-      <c r="D35" t="n">
-        <v>20.47</v>
-      </c>
-      <c r="E35" s="3" t="n">
-        <v>10.16</v>
-      </c>
-      <c r="F35" t="n">
-        <v>1008</v>
-      </c>
-      <c r="G35" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H35" t="n">
-        <v>1871</v>
-      </c>
-      <c r="I35" t="n">
-        <v>1492288</v>
-      </c>
-      <c r="J35" t="n">
-        <v>5.31</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>VICR</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>210</v>
-      </c>
-      <c r="D36" t="n">
-        <v>190.68</v>
-      </c>
-      <c r="E36" s="3" t="n">
-        <v>10.13</v>
-      </c>
-      <c r="F36" t="n">
-        <v>6343</v>
-      </c>
-      <c r="G36" s="3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H36" t="n">
-        <v>7628</v>
-      </c>
-      <c r="I36" t="n">
-        <v>945596</v>
-      </c>
-      <c r="J36" t="n">
-        <v>7.57</v>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>CMPS</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>12.22</v>
-      </c>
-      <c r="D37" t="n">
-        <v>11.11</v>
-      </c>
-      <c r="E37" s="3" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="F37" t="n">
-        <v>7383</v>
-      </c>
-      <c r="G37" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" t="n">
-        <v>7450</v>
-      </c>
-      <c r="I37" t="n">
-        <v>2676118</v>
-      </c>
-      <c r="J37" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>SPHR</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>113</v>
-      </c>
-      <c r="D38" t="n">
-        <v>102.89</v>
-      </c>
-      <c r="E38" s="3" t="n">
-        <v>9.83</v>
-      </c>
-      <c r="F38" t="n">
-        <v>33</v>
-      </c>
-      <c r="G38" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H38" t="n">
-        <v>89</v>
-      </c>
-      <c r="I38" t="n">
-        <v>779264</v>
-      </c>
-      <c r="J38" t="n">
-        <v>5.42</v>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>CGEM</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>15.35</v>
-      </c>
-      <c r="D39" t="n">
-        <v>13.98</v>
-      </c>
-      <c r="E39" s="3" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="F39" t="n">
-        <v>1273</v>
-      </c>
-      <c r="G39" s="3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H39" t="n">
-        <v>2057</v>
-      </c>
-      <c r="I39" t="n">
-        <v>1007690</v>
-      </c>
-      <c r="J39" t="n">
-        <v>7.79</v>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>AKTS</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>16.59</v>
-      </c>
-      <c r="D40" t="n">
-        <v>15.11</v>
-      </c>
-      <c r="E40" s="3" t="n">
-        <v>9.789999999999999</v>
-      </c>
-      <c r="F40" t="n">
-        <v>17</v>
-      </c>
-      <c r="G40" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H40" t="n">
-        <v>60</v>
-      </c>
-      <c r="I40" t="n">
-        <v>390470</v>
-      </c>
-      <c r="J40" t="n">
-        <v>5.39</v>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>GLUE</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="D41" t="n">
-        <v>10.66</v>
-      </c>
-      <c r="E41" s="3" t="n">
-        <v>9.76</v>
-      </c>
-      <c r="F41" t="n">
-        <v>377</v>
-      </c>
-      <c r="G41" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" t="n">
-        <v>11954</v>
-      </c>
-      <c r="I41" t="n">
-        <v>1252232</v>
-      </c>
-      <c r="J41" t="n">
-        <v>5.86</v>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>CLYM</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>10.66</v>
-      </c>
-      <c r="D42" t="n">
-        <v>9.73</v>
-      </c>
-      <c r="E42" s="3" t="n">
-        <v>9.56</v>
-      </c>
-      <c r="F42" t="n">
-        <v>114</v>
-      </c>
-      <c r="G42" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" t="n">
-        <v>9353</v>
-      </c>
-      <c r="I42" t="n">
-        <v>1436500</v>
-      </c>
-      <c r="J42" t="n">
-        <v>6.54</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>SLDB</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>6.48</v>
-      </c>
-      <c r="D43" t="n">
-        <v>5.92</v>
-      </c>
-      <c r="E43" s="3" t="n">
-        <v>9.460000000000001</v>
-      </c>
-      <c r="F43" t="n">
-        <v>430</v>
-      </c>
-      <c r="G43" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H43" t="n">
-        <v>427</v>
-      </c>
-      <c r="I43" t="n">
-        <v>1206210</v>
-      </c>
-      <c r="J43" t="n">
-        <v>6.44</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>TNGX</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>25.74</v>
-      </c>
-      <c r="D44" t="n">
-        <v>23.53</v>
-      </c>
-      <c r="E44" s="3" t="n">
-        <v>9.390000000000001</v>
-      </c>
-      <c r="F44" t="n">
-        <v>12507</v>
-      </c>
-      <c r="G44" s="2" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="H44" t="n">
-        <v>1198</v>
-      </c>
-      <c r="I44" t="n">
-        <v>2966906</v>
-      </c>
-      <c r="J44" t="n">
-        <v>6.86</v>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>IMMX</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="D45" t="n">
-        <v>8.220000000000001</v>
-      </c>
-      <c r="E45" s="3" t="n">
-        <v>9.369999999999999</v>
-      </c>
-      <c r="F45" t="n">
-        <v>532</v>
-      </c>
-      <c r="G45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>13172</v>
-      </c>
-      <c r="I45" t="n">
-        <v>1592550</v>
-      </c>
-      <c r="J45" t="n">
-        <v>7.14</v>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>TRU</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>79.93000000000001</v>
-      </c>
-      <c r="D46" t="n">
-        <v>73.12</v>
-      </c>
-      <c r="E46" s="3" t="n">
-        <v>9.31</v>
-      </c>
-      <c r="F46" t="n">
-        <v>112</v>
-      </c>
-      <c r="G46" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" t="n">
-        <v>2504260</v>
-      </c>
-      <c r="I46" t="n">
-        <v>2504260</v>
-      </c>
-      <c r="J46" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>proxy</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>CRVS</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>10.54</v>
-      </c>
-      <c r="D47" t="n">
-        <v>9.65</v>
-      </c>
-      <c r="E47" s="3" t="n">
-        <v>9.220000000000001</v>
-      </c>
-      <c r="F47" t="n">
-        <v>212</v>
-      </c>
-      <c r="G47" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H47" t="n">
-        <v>519</v>
-      </c>
-      <c r="I47" t="n">
-        <v>1028296</v>
-      </c>
-      <c r="J47" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>SRPT</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>19.36</v>
-      </c>
-      <c r="D48" t="n">
-        <v>17.73</v>
-      </c>
-      <c r="E48" s="3" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="F48" t="n">
-        <v>233</v>
-      </c>
-      <c r="G48" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" t="n">
-        <v>8889</v>
-      </c>
-      <c r="I48" t="n">
-        <v>3042962</v>
-      </c>
-      <c r="J48" t="n">
-        <v>4.78</v>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>RLAY</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>18.65</v>
-      </c>
-      <c r="D49" t="n">
-        <v>17.09</v>
-      </c>
-      <c r="E49" s="3" t="n">
-        <v>9.130000000000001</v>
-      </c>
-      <c r="F49" t="n">
-        <v>623</v>
-      </c>
-      <c r="G49" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H49" t="n">
-        <v>8883</v>
-      </c>
-      <c r="I49" t="n">
-        <v>2941628</v>
-      </c>
-      <c r="J49" t="n">
-        <v>5.37</v>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>EVC</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>6.89</v>
-      </c>
-      <c r="D50" t="n">
-        <v>6.32</v>
-      </c>
-      <c r="E50" s="3" t="n">
-        <v>9.1</v>
-      </c>
-      <c r="F50" t="n">
-        <v>105</v>
-      </c>
-      <c r="G50" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H50" t="n">
-        <v>297</v>
-      </c>
-      <c r="I50" t="n">
-        <v>1428844</v>
-      </c>
-      <c r="J50" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>CHPT</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="D51" t="n">
-        <v>7.15</v>
-      </c>
-      <c r="E51" s="3" t="n">
-        <v>9.09</v>
-      </c>
-      <c r="F51" t="n">
-        <v>3451</v>
-      </c>
-      <c r="G51" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H51" t="n">
-        <v>27620</v>
-      </c>
-      <c r="I51" t="n">
-        <v>2156410</v>
-      </c>
-      <c r="J51" t="n">
-        <v>7.52</v>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>MGTX</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="D52" t="n">
-        <v>9.449999999999999</v>
-      </c>
-      <c r="E52" s="3" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="F52" t="n">
-        <v>87</v>
-      </c>
-      <c r="G52" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H52" t="n">
-        <v>844</v>
-      </c>
-      <c r="I52" t="n">
-        <v>878162</v>
-      </c>
-      <c r="J52" t="n">
-        <v>5.49</v>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>STOK</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>26.99</v>
-      </c>
-      <c r="D53" t="n">
-        <v>24.82</v>
-      </c>
-      <c r="E53" s="3" t="n">
-        <v>8.74</v>
-      </c>
-      <c r="F53" t="n">
-        <v>585</v>
-      </c>
-      <c r="G53" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H53" t="n">
-        <v>1851</v>
-      </c>
-      <c r="I53" t="n">
-        <v>883578</v>
-      </c>
-      <c r="J53" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>COMP</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>9.789999999999999</v>
-      </c>
-      <c r="D54" t="n">
-        <v>9.01</v>
-      </c>
-      <c r="E54" s="3" t="n">
-        <v>8.66</v>
-      </c>
-      <c r="F54" t="n">
-        <v>10782</v>
-      </c>
-      <c r="G54" s="2" t="n">
-        <v>21.1</v>
-      </c>
-      <c r="H54" t="n">
-        <v>509</v>
-      </c>
-      <c r="I54" t="n">
-        <v>13410634</v>
-      </c>
-      <c r="J54" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>VSTM</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>9.359999999999999</v>
-      </c>
-      <c r="D55" t="n">
-        <v>8.619999999999999</v>
-      </c>
-      <c r="E55" s="3" t="n">
-        <v>8.58</v>
-      </c>
-      <c r="F55" t="n">
-        <v>3011</v>
-      </c>
-      <c r="G55" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" t="n">
-        <v>91836</v>
-      </c>
-      <c r="I55" t="n">
-        <v>3339552</v>
-      </c>
-      <c r="J55" t="n">
-        <v>8.710000000000001</v>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>8.859999999999999</v>
-      </c>
-      <c r="D56" t="n">
-        <v>8.16</v>
-      </c>
-      <c r="E56" s="3" t="n">
-        <v>8.58</v>
-      </c>
-      <c r="F56" t="n">
-        <v>117733</v>
-      </c>
-      <c r="G56" s="3" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="H56" t="n">
-        <v>103452</v>
-      </c>
-      <c r="I56" t="n">
-        <v>13734216</v>
-      </c>
-      <c r="J56" t="n">
-        <v>6.46</v>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>ASST</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>27.72</v>
-      </c>
-      <c r="D57" t="n">
-        <v>25.54</v>
-      </c>
-      <c r="E57" s="3" t="n">
-        <v>8.539999999999999</v>
-      </c>
-      <c r="F57" t="n">
-        <v>79519</v>
-      </c>
-      <c r="G57" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H57" t="n">
-        <v>233684</v>
-      </c>
-      <c r="I57" t="n">
-        <v>9010294</v>
-      </c>
-      <c r="J57" t="n">
-        <v>5.97</v>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>IMTX</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>7.65</v>
-      </c>
-      <c r="D58" t="n">
-        <v>7.05</v>
-      </c>
-      <c r="E58" s="3" t="n">
-        <v>8.51</v>
-      </c>
-      <c r="F58" t="n">
-        <v>22</v>
-      </c>
-      <c r="G58" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" t="n">
-        <v>1899</v>
-      </c>
-      <c r="I58" t="n">
-        <v>768838</v>
-      </c>
-      <c r="J58" t="n">
-        <v>5.65</v>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>RVMD</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>197.46</v>
-      </c>
-      <c r="D59" t="n">
-        <v>182.15</v>
-      </c>
-      <c r="E59" s="3" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="F59" t="n">
-        <v>348</v>
-      </c>
-      <c r="G59" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" t="n">
-        <v>2013772</v>
-      </c>
-      <c r="I59" t="n">
-        <v>2013772</v>
-      </c>
-      <c r="J59" t="n">
-        <v>4.54</v>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>proxy</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>DMRA</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>20.88</v>
-      </c>
-      <c r="D60" t="n">
-        <v>19.27</v>
-      </c>
-      <c r="E60" s="3" t="n">
-        <v>8.35</v>
-      </c>
-      <c r="F60" t="n">
-        <v>2</v>
-      </c>
-      <c r="G60" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" t="n">
-        <v>254</v>
-      </c>
-      <c r="I60" t="n">
-        <v>552400</v>
-      </c>
-      <c r="J60" t="n">
-        <v>6.99</v>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>BMNR</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>23.35</v>
-      </c>
-      <c r="D61" t="n">
-        <v>21.57</v>
-      </c>
-      <c r="E61" s="3" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="F61" t="n">
-        <v>340178</v>
-      </c>
-      <c r="G61" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H61" t="n">
-        <v>874166</v>
-      </c>
-      <c r="I61" t="n">
-        <v>39073798</v>
-      </c>
-      <c r="J61" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>DELL</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>492.15</v>
-      </c>
-      <c r="D62" t="n">
-        <v>454.81</v>
-      </c>
-      <c r="E62" s="3" t="n">
-        <v>8.210000000000001</v>
-      </c>
-      <c r="F62" t="n">
-        <v>123074</v>
-      </c>
-      <c r="G62" s="3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="H62" t="n">
-        <v>102647</v>
-      </c>
-      <c r="I62" t="n">
-        <v>8088102</v>
-      </c>
-      <c r="J62" t="n">
-        <v>4.65</v>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>TDOC</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="D63" t="n">
-        <v>5.73</v>
-      </c>
-      <c r="E63" s="3" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="F63" t="n">
-        <v>1067</v>
-      </c>
-      <c r="G63" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H63" t="n">
-        <v>3518374</v>
-      </c>
-      <c r="I63" t="n">
-        <v>3518374</v>
-      </c>
-      <c r="J63" t="n">
-        <v>4.03</v>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>proxy</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>STTK</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>5.81</v>
-      </c>
-      <c r="D64" t="n">
-        <v>5.37</v>
-      </c>
-      <c r="E64" s="3" t="n">
-        <v>8.19</v>
-      </c>
-      <c r="F64" t="n">
-        <v>16</v>
-      </c>
-      <c r="G64" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H64" t="n">
-        <v>250</v>
-      </c>
-      <c r="I64" t="n">
-        <v>1193606</v>
-      </c>
-      <c r="J64" t="n">
-        <v>7.61</v>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>SOPH</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>7.02</v>
-      </c>
-      <c r="D65" t="n">
-        <v>6.49</v>
-      </c>
-      <c r="E65" s="3" t="n">
-        <v>8.17</v>
-      </c>
-      <c r="F65" t="n">
-        <v>124</v>
-      </c>
-      <c r="G65" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H65" t="n">
-        <v>542</v>
-      </c>
-      <c r="I65" t="n">
-        <v>624164</v>
-      </c>
-      <c r="J65" t="n">
-        <v>6.53</v>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>ALMR</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>28.45</v>
-      </c>
-      <c r="D66" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="E66" s="3" t="n">
-        <v>8.16</v>
-      </c>
-      <c r="F66" t="n">
-        <v>100</v>
-      </c>
-      <c r="G66" s="3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H66" t="n">
-        <v>179</v>
-      </c>
-      <c r="I66" t="n">
-        <v>544326</v>
-      </c>
-      <c r="J66" t="n">
-        <v>9.119999999999999</v>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>AURA</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="D67" t="n">
-        <v>6.29</v>
-      </c>
-      <c r="E67" s="3" t="n">
-        <v>8.109999999999999</v>
-      </c>
-      <c r="F67" t="n">
-        <v>34</v>
-      </c>
-      <c r="G67" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H67" t="n">
-        <v>191</v>
-      </c>
-      <c r="I67" t="n">
-        <v>925192</v>
-      </c>
-      <c r="J67" t="n">
-        <v>4.23</v>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>SBET</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>8.06</v>
-      </c>
-      <c r="D68" t="n">
-        <v>7.46</v>
-      </c>
-      <c r="E68" s="3" t="n">
-        <v>8.039999999999999</v>
-      </c>
-      <c r="F68" t="n">
-        <v>24963</v>
-      </c>
-      <c r="G68" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H68" t="n">
-        <v>58295</v>
-      </c>
-      <c r="I68" t="n">
-        <v>8675302</v>
-      </c>
-      <c r="J68" t="n">
-        <v>5.44</v>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>CMCT</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>5.66</v>
-      </c>
-      <c r="D69" t="n">
-        <v>5.24</v>
-      </c>
-      <c r="E69" s="3" t="n">
-        <v>8.02</v>
-      </c>
-      <c r="F69" t="n">
-        <v>22</v>
-      </c>
-      <c r="G69" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" t="n">
-        <v>717660</v>
-      </c>
-      <c r="I69" t="n">
-        <v>717660</v>
-      </c>
-      <c r="J69" t="n">
-        <v>19.22</v>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>proxy</t>
         </is>
       </c>
     </row>
@@ -3529,7 +1501,7 @@
         <v>7453792</v>
       </c>
       <c r="L3" t="n">
-        <v>5427718</v>
+        <v>5428812</v>
       </c>
       <c r="M3" t="n">
         <v>12.33</v>
@@ -3959,7 +1931,7 @@
         <v>6505884</v>
       </c>
       <c r="L8" t="n">
-        <v>2800361</v>
+        <v>2800947</v>
       </c>
       <c r="M8" t="n">
         <v>11.72</v>
@@ -3987,7 +1959,7 @@
         <v>-15.3</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>57</v>
+        <v>56.9</v>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
@@ -4045,7 +2017,7 @@
         <v>23992636</v>
       </c>
       <c r="L9" t="n">
-        <v>18497925</v>
+        <v>18500168</v>
       </c>
       <c r="M9" t="n">
         <v>220.85</v>
@@ -4131,7 +2103,7 @@
         <v>18876917</v>
       </c>
       <c r="L10" t="n">
-        <v>13852586</v>
+        <v>13854393</v>
       </c>
       <c r="M10" t="n">
         <v>14.11</v>
@@ -4389,7 +2361,7 @@
         <v>7989739</v>
       </c>
       <c r="L13" t="n">
-        <v>8465773</v>
+        <v>8467410</v>
       </c>
       <c r="M13" t="n">
         <v>26.65</v>
@@ -4733,7 +2705,7 @@
         <v>3924275</v>
       </c>
       <c r="L17" t="n">
-        <v>3384242</v>
+        <v>3385857</v>
       </c>
       <c r="M17" t="n">
         <v>10.87</v>
@@ -4761,7 +2733,7 @@
         <v>-31</v>
       </c>
       <c r="T17" s="2" t="n">
-        <v>13.8</v>
+        <v>13.7</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -6120,7 +4092,7 @@
         <v>10.9</v>
       </c>
       <c r="U11" t="n">
-        <v>-7.9</v>
+        <v>-8</v>
       </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="n">
@@ -6605,7 +4577,7 @@
         <v>30.17</v>
       </c>
       <c r="U16" t="n">
-        <v>12.7</v>
+        <v>12.6</v>
       </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="n">
@@ -9941,7 +7913,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>105.54</v>
+        <v>105.36</v>
       </c>
       <c r="D19" t="n">
         <v>2</v>
@@ -9961,7 +7933,7 @@
         <v>97.63</v>
       </c>
       <c r="I19" t="n">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
@@ -9969,7 +7941,7 @@
         </is>
       </c>
       <c r="K19" s="2" t="n">
-        <v>12.7</v>
+        <v>17.3</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
@@ -9982,25 +7954,25 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>95.61</v>
+        <v>95.93000000000001</v>
       </c>
       <c r="O19" t="n">
-        <v>88.95</v>
+        <v>89.04000000000001</v>
       </c>
       <c r="P19" t="n">
-        <v>85.93000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="Q19" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="R19" t="n">
-        <v>6205547</v>
+        <v>6214644</v>
       </c>
       <c r="S19" t="n">
-        <v>13.2</v>
+        <v>12.2</v>
       </c>
       <c r="T19" t="n">
-        <v>21.3</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="20">
@@ -10473,7 +8445,7 @@
         </is>
       </c>
       <c r="K26" s="2" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
@@ -10805,7 +8777,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>52.28</v>
+        <v>52.04</v>
       </c>
       <c r="D31" t="n">
         <v>2</v>
@@ -10825,7 +8797,7 @@
         <v>49.63</v>
       </c>
       <c r="I31" t="n">
-        <v>5.3</v>
+        <v>4.9</v>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
@@ -10833,7 +8805,7 @@
         </is>
       </c>
       <c r="K31" s="2" t="n">
-        <v>22.6</v>
+        <v>27.6</v>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
@@ -10846,25 +8818,25 @@
         </is>
       </c>
       <c r="N31" t="n">
-        <v>49.84</v>
+        <v>49.9</v>
       </c>
       <c r="O31" t="n">
-        <v>45.72</v>
+        <v>45.82</v>
       </c>
       <c r="P31" t="n">
-        <v>41.98</v>
+        <v>42.09</v>
       </c>
       <c r="Q31" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="R31" t="n">
-        <v>486714</v>
+        <v>479652</v>
       </c>
       <c r="S31" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="T31" t="n">
-        <v>6.5</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="32">
@@ -12672,7 +10644,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>52.28</v>
+        <v>52.04</v>
       </c>
       <c r="E8" t="n">
         <v>46.17</v>
@@ -12711,22 +10683,22 @@
         <v>50.77</v>
       </c>
       <c r="Q8" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.83</v>
+        <v>0.7</v>
       </c>
       <c r="S8" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="T8" t="n">
-        <v>486714</v>
+        <v>479652</v>
       </c>
       <c r="U8" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="V8" t="n">
-        <v>6.5</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="9">
@@ -13362,7 +11334,7 @@
         <v>-4.4</v>
       </c>
       <c r="R17" s="2" t="n">
-        <v>1.84</v>
+        <v>1.86</v>
       </c>
       <c r="S17" t="n">
         <v>6.56</v>
@@ -14514,7 +12486,7 @@
         <v>-14.8</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="S33" t="n">
         <v>4.48</v>
@@ -16890,7 +14862,7 @@
         <v>-14</v>
       </c>
       <c r="R66" s="3" t="n">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="S66" t="n">
         <v>4.03</v>
@@ -18154,7 +16126,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-21 20:51:39</t>
+          <t>2026-10-22 20:51:40</t>
         </is>
       </c>
     </row>
@@ -18165,7 +16137,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4566</v>
+        <v>4578</v>
       </c>
     </row>
     <row r="3">
@@ -18175,7 +16147,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>68</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -18256,7 +16228,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>284s</t>
+          <t>286s</t>
         </is>
       </c>
     </row>

</xml_diff>